<commit_message>
Add CF1_8wcon as the representative CF slide at 8wcon
Completes the representative-slide list so every post-lesion participant and
timepoint has a select slide.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Post_heal_representative_slides_10132026.xlsx
+++ b/Post_heal_representative_slides_10132026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kphasouk/Desktop/HSV406/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93AE2D4A-9988-A14D-89EF-147BE5B7C3AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B2A1A2E-7E2D-B44D-9958-569857956649}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13580" yWindow="7980" windowWidth="26040" windowHeight="14680" xr2:uid="{4E01D0DD-8A4D-2245-9244-13741CD5B95B}"/>
+    <workbookView xWindow="13580" yWindow="7960" windowWidth="26040" windowHeight="14680" xr2:uid="{4E01D0DD-8A4D-2245-9244-13741CD5B95B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>CF2_2wph</t>
   </si>
@@ -84,6 +84,9 @@
   </si>
   <si>
     <t>SK1_8wph</t>
+  </si>
+  <si>
+    <t>CF1_8wcon</t>
   </si>
 </sst>
 </file>
@@ -455,7 +458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6F4288A-E383-EC42-9701-89A12A15E5A2}">
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
@@ -465,71 +468,76 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>